<commit_message>
feat: packs autosuficientes - cada estrategia trae TODAS sus senales
base_senales.xlsx eliminado: cada <pack>_senales.xlsx incluye todas las
senales que su estrategia usa (componentes + dependencias de composites),
duplicando las compartidas - el import upsertea por key, asi que no hay
conflicto y el orden entre packs deja de importar.

- pullback: + rsi_senal, tendencia_d
- momentum: + fuerza_relativa_52w, alineacion_timeframes,
  tendencia_d/w/m, dist_sma_d (ya no requiere importar pullback antes)
- garp: + tendencia_m
- pullback_bajista: + dist_sma_d

test_strategy_packs endurecido: cada estrategia se valida contra SU
propio excel de senales (autosuficiencia real), y las refs de composites
deben resolverse dentro del mismo archivo.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/strategy_packs/garp_senales.xlsx
+++ b/strategy_packs/garp_senales.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,7 +471,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Retorno sobre capital invertido (TTM, fracción): &gt;20% → 100; &gt;10% → 60; &gt;5% → 20; positivo → −20; negativo/sin dato → −80.</t>
+          <t>Retorno sobre capital invertido (TTM, fraccion): &gt;20% -&gt; 100; &gt;10% -&gt; 60; &gt;5% -&gt; 20; positivo -&gt; -20; negativo/sin dato -&gt; -80.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -509,7 +509,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Premia P/E TTM bajo pero positivo: &lt;8 → 100; 8-15 → 80; 15-25 → 30; 25-40 → −30; &gt;40 → −80; negativo (pérdidas) → −100.</t>
+          <t>Premia P/E TTM bajo pero positivo: &lt;8 -&gt; 100; 8-15 -&gt; 80; 15-25 -&gt; 30; 25-40 -&gt; -30; &gt;40 -&gt; -80; negativo (perdidas) -&gt; -100.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Crecimiento de revenue interanual (fracción) mapeado lineal: −10% → −100; +10% → 0; +30% o más → +100.</t>
+          <t>Crecimiento de revenue interanual (fraccion) mapeado lineal: -10% -&gt; -100; +10% -&gt; 0; +30% o mas -&gt; +100.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -569,6 +569,44 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>{"min": -0.1, "max": 0.3, "clamp": true}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tendencia_m</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tendencia mensual</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Mapa del regimen de tendencia mensual a score.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>asset</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>trend_monthly</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>discrete_map</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>{"map": {"bullish_strong": 100, "bullish_nascent_strong": 75, "bullish": 60, "bullish_nascent": 40, "lateral_nascent": 5, "lateral": 0, "bearish_nascent": -40, "bearish_nascent_strong": -75, "bearish": -60, "bearish_strong": -100}}</t>
         </is>
       </c>
     </row>

</xml_diff>